<commit_message>
Usar el equipo de finanzas real en el Excel del organigrama
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WWpepS9wV9DZhmZr7JVMkV
</commit_message>
<xml_diff>
--- a/organigrama/Organigrama.xlsx
+++ b/organigrama/Organigrama.xlsx
@@ -129,8 +129,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Organigrama" displayName="Organigrama" ref="A1:G13" headerRowCount="1">
-  <autoFilter ref="A1:G13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Organigrama" displayName="Organigrama" ref="A1:G9" headerRowCount="1">
+  <autoFilter ref="A1:G9"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Nombre"/>
     <tableColumn id="2" name="Puesto"/>
@@ -433,16 +433,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="80" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -485,12 +485,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Laura Méndez</t>
+          <t>Chris F</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Directora General</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -500,425 +500,245 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>laura.mendez@empresa.com</t>
+          <t>chris.f@empresa.com</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>55 1000 0001</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Define la estrategia de la empresa y lidera al equipo directivo. Más de 15 años en el sector.</t>
+          <t>Lidera la empresa y define la estrategia general.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Carlos Ruiz</t>
+          <t>Vern Fleming</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Director de Ventas</t>
+          <t>President</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Ventas</t>
+          <t>Dirección</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>carlos.ruiz@empresa.com</t>
+          <t>vern.fleming@empresa.com</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>laura.mendez@empresa.com</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>55 1000 0002</t>
-        </is>
-      </c>
+          <t>chris.f@empresa.com</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Responsable de las metas comerciales, clientes clave y expansión a nuevos mercados.</t>
+          <t>Dirige la operación de la empresa y supervisa a las áreas clave.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ana Torres</t>
+          <t>Jessica Zaap</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Directora de Operaciones</t>
+          <t>VP Finance</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Operaciones</t>
+          <t>Finanzas</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ana.torres@empresa.com</t>
+          <t>jessica.zaap@empresa.com</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>laura.mendez@empresa.com</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>55 1000 0003</t>
-        </is>
-      </c>
+          <t>vern.fleming@empresa.com</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Coordina logística, inventarios y procesos para que todo llegue a tiempo.</t>
+          <t>Responsable del área de finanzas y de recursos humanos.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Miguel Ángel Soto</t>
+          <t>Emily K</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Director de Finanzas</t>
+          <t>HR Manager</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Finanzas</t>
+          <t>Recursos Humanos</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>miguel.soto@empresa.com</t>
+          <t>emily.k@empresa.com</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>laura.mendez@empresa.com</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>55 1000 0004</t>
-        </is>
-      </c>
+          <t>jessica.zaap@empresa.com</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Lleva presupuestos, flujo de caja y reportes financieros.</t>
+          <t>Gestiona contratación, nómina y desarrollo del personal.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sofía Herrera</t>
+          <t>Vacante</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Gerente de Marketing</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Finanzas</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>sofia.herrera@empresa.com</t>
+          <t>vacante.finanzas@empresa.com</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>laura.mendez@empresa.com</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>55 1000 0005</t>
-        </is>
-      </c>
+          <t>jessica.zaap@empresa.com</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Marca, redes sociales y campañas. Le encanta probar ideas nuevas.</t>
+          <t>Posición abierta en el equipo de finanzas.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Diego Castillo</t>
+          <t>Jennifer B</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ejecutivo de Ventas</t>
+          <t>CFO</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Ventas</t>
+          <t>Finanzas</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>diego.castillo@empresa.com</t>
+          <t>jennifer.b@empresa.com</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>carlos.ruiz@empresa.com</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>55 1000 0006</t>
-        </is>
-      </c>
+          <t>jessica.zaap@empresa.com</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Atiende cuentas de la zona norte y prospecta nuevos clientes.</t>
+          <t>Lleva la estrategia financiera, presupuestos y reportes.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Valeria Gómez</t>
+          <t>Cindy F</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ejecutiva de Ventas</t>
+          <t>Accounting</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Ventas</t>
+          <t>Finanzas</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>valeria.gomez@empresa.com</t>
+          <t>cindy.f@empresa.com</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>carlos.ruiz@empresa.com</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>55 1000 0007</t>
-        </is>
-      </c>
+          <t>jennifer.b@empresa.com</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Atiende cuentas corporativas y da seguimiento a cotizaciones.</t>
+          <t>Contabilidad, cierres mensuales y conciliaciones.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Jorge Navarro</t>
+          <t>Alice</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Coordinador de Logística</t>
+          <t>Assistant</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Operaciones</t>
+          <t>Finanzas</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>jorge.navarro@empresa.com</t>
+          <t>alice@empresa.com</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ana.torres@empresa.com</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>55 1000 0008</t>
-        </is>
-      </c>
+          <t>jennifer.b@empresa.com</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Programa envíos y coordina con proveedores de transporte.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Paola Ríos</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Analista de Inventarios</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Operaciones</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>paola.rios@empresa.com</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>ana.torres@empresa.com</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>55 1000 0009</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Controla existencias y prepara reportes semanales de inventario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Ricardo Vega</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Contador</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Finanzas</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>ricardo.vega@empresa.com</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>miguel.soto@empresa.com</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>55 1000 0010</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Contabilidad, impuestos y conciliaciones bancarias.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Fernanda Luna</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Diseñadora Gráfica</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>fernanda.luna@empresa.com</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>sofia.herrera@empresa.com</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>55 1000 0011</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Crea piezas visuales para redes, catálogos y presentaciones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Andrés Molina</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Community Manager</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>andres.molina@empresa.com</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>sofia.herrera@empresa.com</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>55 1000 0012</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Gestiona redes sociales y responde a la comunidad.</t>
+          <t>Apoyo administrativo al equipo de finanzas.</t>
         </is>
       </c>
     </row>

</xml_diff>